<commit_message>
fix(excel): open PS export without Excel repair dialog
Remove sheetView pageBreakPreview from the stripped blank (Excel refuses
the package) and clear Dart zip UTF-8 flags; keep contrast fonts and 1x1 print.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/assets/templates/ps_weekly_blank.xlsx
+++ b/assets/templates/ps_weekly_blank.xlsx
@@ -4,9 +4,6 @@
   <sheets>
     <sheet name="Settimana" sheetId="1" r:id="rId1"/>
   </sheets>
-  <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'Settimana'!$A$1:$O$70</definedName>
-  </definedNames>
 </workbook>
 </file>
 
@@ -3019,7 +3016,6 @@
       <family val="2"/>
     </font>
     <font>
-      <!-- corsi-white -->
       <b/>
       <sz val="8"/>
       <color rgb="FFFFFFFF"/>
@@ -3027,7 +3023,6 @@
       <family val="2"/>
     </font>
     <font>
-      <!-- corsi-dark -->
       <b/>
       <sz val="8"/>
       <color rgb="FF111827"/>
@@ -10432,7 +10427,6 @@
     <xf numFmtId="1" fontId="71" fillId="0" borderId="4" xfId="29" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
     </xf>
-    <!-- corsi-module-xfs -->
     <xf numFmtId="0" fontId="109" fillId="82" borderId="137" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
     </xf>
@@ -12581,13 +12575,13 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{368E55A2-AD71-4714-92B2-F8C5DEE7E7F4}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheetPr>
     <tabColor rgb="FF00B0F0"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:AG65"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <dimension ref="A1:O70"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="12.75"/>
   <cols>
     <col min="1" max="1" width="3" style="421" customWidth="1"/>
     <col min="2" max="2" width="11" style="421" bestFit="1" customWidth="1"/>
@@ -12605,12 +12599,12 @@
     <col min="17" max="16384" width="9.140625" style="421"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:33" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:33" ht="15" customHeight="1" thickBot="1">
       <c r="A1" s="421" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:33" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:33" ht="15" customHeight="1">
       <c r="B2" s="1258" t="s">
         <v>0</v>
       </c>
@@ -12631,7 +12625,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:33" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:33" ht="15" customHeight="1">
       <c r="B3" s="1261" t="s">
         <v>9</v>
       </c>
@@ -12649,7 +12643,7 @@
       <c r="N3" s="1262"/>
       <c r="O3" s="1263"/>
     </row>
-    <row r="4" spans="1:33" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:33" ht="15" customHeight="1">
       <c r="B4" s="1261" t="s">
         <v>652</v>
       </c>
@@ -12667,7 +12661,7 @@
       <c r="N4" s="1262"/>
       <c r="O4" s="1263"/>
     </row>
-    <row r="5" spans="1:33" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:33" ht="15" customHeight="1" thickBot="1">
       <c r="B5" s="1264" t="inlineStr">
         <is>
           <t>{{COURSE_TITLE}}</t>
@@ -12687,7 +12681,7 @@
       <c r="N5" s="1265"/>
       <c r="O5" s="1266"/>
     </row>
-    <row r="6" spans="1:33" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:33" ht="15" customHeight="1" thickBot="1">
       <c r="B6" s="683" t="s">
         <v>11</v>
       </c>
@@ -12707,7 +12701,7 @@
       <c r="N6" s="1070"/>
       <c r="O6" s="1071"/>
     </row>
-    <row r="7" spans="1:33" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:33" ht="15" customHeight="1" thickBot="1">
       <c r="B7" s="690" t="s">
         <v>1</v>
       </c>
@@ -12727,7 +12721,7 @@
       <c r="N7" s="1073"/>
       <c r="O7" s="1074"/>
     </row>
-    <row r="8" spans="1:33" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:33" ht="15" customHeight="1">
       <c r="B8" s="699" t="s">
         <v>2</v>
       </c>
@@ -12776,7 +12770,7 @@
       <c r="AF8" s="531"/>
       <c r="AG8" s="531"/>
     </row>
-    <row r="9" spans="1:33" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:33" ht="15" customHeight="1" thickBot="1">
       <c r="B9" s="700"/>
       <c r="C9" s="702"/>
       <c r="D9" s="703"/>
@@ -12802,7 +12796,7 @@
       <c r="AF9" s="531"/>
       <c r="AG9" s="531"/>
     </row>
-    <row r="10" spans="1:33" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:33" ht="15" customHeight="1">
       <c r="B10" s="613"/>
       <c r="C10" s="539" t="s">
         <v>67</v>
@@ -12826,7 +12820,7 @@
       <c r="AF10" s="531"/>
       <c r="AG10" s="531"/>
     </row>
-    <row r="11" spans="1:33" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:33" ht="15" customHeight="1">
       <c r="B11" s="614"/>
       <c r="C11" s="547" t="s">
         <v>643</v>
@@ -12861,7 +12855,7 @@
       <c r="AF11" s="531"/>
       <c r="AG11" s="531"/>
     </row>
-    <row r="12" spans="1:33" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:33" ht="15" customHeight="1">
       <c r="B12" s="614"/>
       <c r="C12" s="547" t="s">
         <v>644</v>
@@ -12894,7 +12888,7 @@
       <c r="AF12" s="531"/>
       <c r="AG12" s="531"/>
     </row>
-    <row r="13" spans="1:33" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:33" ht="15" customHeight="1">
       <c r="B13" s="614"/>
       <c r="C13" s="547" t="s">
         <v>645</v>
@@ -12928,7 +12922,7 @@
       <c r="AF13" s="531"/>
       <c r="AG13" s="531"/>
     </row>
-    <row r="14" spans="1:33" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:33" ht="15" customHeight="1">
       <c r="B14" s="614"/>
       <c r="C14" s="547" t="s">
         <v>670</v>
@@ -12949,7 +12943,7 @@
       <c r="AA14" s="531"/>
       <c r="AB14" s="531"/>
     </row>
-    <row r="15" spans="1:33" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:33" ht="15" customHeight="1">
       <c r="B15" s="614"/>
       <c r="C15" s="540" t="s">
         <v>671</v>
@@ -12974,7 +12968,7 @@
       <c r="AF15" s="531"/>
       <c r="AG15" s="531"/>
     </row>
-    <row r="16" spans="1:33" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:33" ht="15" customHeight="1">
       <c r="B16" s="614"/>
       <c r="C16" s="547" t="s">
         <v>649</v>
@@ -12999,7 +12993,7 @@
       <c r="AF16" s="531"/>
       <c r="AG16" s="531"/>
     </row>
-    <row r="17" spans="2:33" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="2:33" ht="15" customHeight="1" thickBot="1">
       <c r="B17" s="615"/>
       <c r="C17" s="548" t="s">
         <v>74</v>
@@ -13025,7 +13019,7 @@
       <c r="AF17" s="531"/>
       <c r="AG17" s="531"/>
     </row>
-    <row r="18" spans="2:33" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="18" spans="2:33" ht="15" customHeight="1">
       <c r="B18" s="613"/>
       <c r="C18" s="549" t="s">
         <v>67</v>
@@ -13049,7 +13043,7 @@
       <c r="AF18" s="531"/>
       <c r="AG18" s="531"/>
     </row>
-    <row r="19" spans="2:33" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="19" spans="2:33" ht="15" customHeight="1">
       <c r="B19" s="614"/>
       <c r="C19" s="547" t="s">
         <v>643</v>
@@ -13074,7 +13068,7 @@
       <c r="AF19" s="531"/>
       <c r="AG19" s="531"/>
     </row>
-    <row r="20" spans="2:33" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="20" spans="2:33" ht="15" customHeight="1">
       <c r="B20" s="614"/>
       <c r="C20" s="547" t="s">
         <v>644</v>
@@ -13095,7 +13089,7 @@
       <c r="AB20" s="531"/>
       <c r="AC20" s="531"/>
     </row>
-    <row r="21" spans="2:33" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="21" spans="2:33" ht="15" customHeight="1">
       <c r="B21" s="614"/>
       <c r="C21" s="547" t="s">
         <v>645</v>
@@ -13116,7 +13110,7 @@
       <c r="AB21" s="531"/>
       <c r="AC21" s="531"/>
     </row>
-    <row r="22" spans="2:33" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="22" spans="2:33" ht="15" customHeight="1">
       <c r="B22" s="614"/>
       <c r="C22" s="547" t="s">
         <v>670</v>
@@ -13138,7 +13132,7 @@
       <c r="AB22" s="531"/>
       <c r="AC22" s="531"/>
     </row>
-    <row r="23" spans="2:33" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="23" spans="2:33" ht="15" customHeight="1">
       <c r="B23" s="614"/>
       <c r="C23" s="550" t="s">
         <v>671</v>
@@ -13166,7 +13160,7 @@
       <c r="AA23" s="531"/>
       <c r="AB23" s="531"/>
     </row>
-    <row r="24" spans="2:33" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="24" spans="2:33" ht="15" customHeight="1">
       <c r="B24" s="614"/>
       <c r="C24" s="547" t="s">
         <v>649</v>
@@ -13194,7 +13188,7 @@
       <c r="AA24" s="531"/>
       <c r="AB24" s="531"/>
     </row>
-    <row r="25" spans="2:33" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="2:33" ht="15" customHeight="1" thickBot="1">
       <c r="B25" s="615"/>
       <c r="C25" s="548" t="s">
         <v>74</v>
@@ -13214,7 +13208,7 @@
       <c r="P25" s="531"/>
       <c r="S25" s="531"/>
     </row>
-    <row r="26" spans="2:33" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="26" spans="2:33" ht="15" customHeight="1">
       <c r="B26" s="613"/>
       <c r="C26" s="549" t="s">
         <v>67</v>
@@ -13243,7 +13237,7 @@
       <c r="AA26" s="531"/>
       <c r="AB26" s="531"/>
     </row>
-    <row r="27" spans="2:33" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="27" spans="2:33" ht="15" customHeight="1">
       <c r="B27" s="614"/>
       <c r="C27" s="554" t="s">
         <v>643</v>
@@ -13262,7 +13256,7 @@
       <c r="O27" s="1231"/>
       <c r="Q27" s="531"/>
     </row>
-    <row r="28" spans="2:33" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="28" spans="2:33" ht="15" customHeight="1">
       <c r="B28" s="614"/>
       <c r="C28" s="554" t="s">
         <v>644</v>
@@ -13282,7 +13276,7 @@
       <c r="P28" s="531"/>
       <c r="Q28" s="531"/>
     </row>
-    <row r="29" spans="2:33" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="29" spans="2:33" ht="15" customHeight="1">
       <c r="B29" s="614"/>
       <c r="C29" s="554" t="s">
         <v>645</v>
@@ -13311,7 +13305,7 @@
       <c r="AA29" s="531"/>
       <c r="AB29" s="531"/>
     </row>
-    <row r="30" spans="2:33" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="30" spans="2:33" ht="15" customHeight="1">
       <c r="B30" s="614"/>
       <c r="C30" s="554" t="s">
         <v>670</v>
@@ -13331,7 +13325,7 @@
       <c r="P30" s="531"/>
       <c r="S30" s="531"/>
     </row>
-    <row r="31" spans="2:33" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="31" spans="2:33" ht="15" customHeight="1">
       <c r="B31" s="614"/>
       <c r="C31" s="583" t="s">
         <v>671</v>
@@ -13351,7 +13345,7 @@
       <c r="Q31" s="531"/>
       <c r="S31" s="531"/>
     </row>
-    <row r="32" spans="2:33" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="32" spans="2:33" ht="15" customHeight="1">
       <c r="B32" s="614"/>
       <c r="C32" s="554" t="s">
         <v>649</v>
@@ -13371,7 +13365,7 @@
       <c r="Q32" s="531"/>
       <c r="AB32" s="531"/>
     </row>
-    <row r="33" spans="1:29" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:29" ht="15" customHeight="1" thickBot="1">
       <c r="B33" s="615"/>
       <c r="C33" s="561" t="s">
         <v>74</v>
@@ -13392,7 +13386,7 @@
       <c r="Q33" s="531"/>
       <c r="AB33" s="531"/>
     </row>
-    <row r="34" spans="1:29" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:29" ht="15" customHeight="1">
       <c r="B34" s="613"/>
       <c r="C34" s="549" t="s">
         <v>67</v>
@@ -13422,7 +13416,7 @@
       <c r="AA34" s="531"/>
       <c r="AB34" s="531"/>
     </row>
-    <row r="35" spans="1:29" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:29" ht="15" customHeight="1">
       <c r="B35" s="614"/>
       <c r="C35" s="547" t="s">
         <v>643</v>
@@ -13452,7 +13446,7 @@
       <c r="AA35" s="531"/>
       <c r="AB35" s="531"/>
     </row>
-    <row r="36" spans="1:29" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:29" ht="15" customHeight="1">
       <c r="B36" s="614"/>
       <c r="C36" s="547" t="s">
         <v>644</v>
@@ -13483,7 +13477,7 @@
       <c r="AA36" s="531"/>
       <c r="AB36" s="531"/>
     </row>
-    <row r="37" spans="1:29" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:29" ht="15" customHeight="1">
       <c r="B37" s="614"/>
       <c r="C37" s="547" t="s">
         <v>645</v>
@@ -13513,7 +13507,7 @@
       <c r="AA37" s="531"/>
       <c r="AB37" s="531"/>
     </row>
-    <row r="38" spans="1:29" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:29" ht="15" customHeight="1">
       <c r="B38" s="614"/>
       <c r="C38" s="554" t="s">
         <v>670</v>
@@ -13543,7 +13537,7 @@
       <c r="AA38" s="531"/>
       <c r="AB38" s="531"/>
     </row>
-    <row r="39" spans="1:29" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:29" ht="15" customHeight="1">
       <c r="B39" s="614"/>
       <c r="C39" s="550" t="s">
         <v>671</v>
@@ -13562,7 +13556,7 @@
       <c r="O39" s="1231"/>
       <c r="AB39" s="531"/>
     </row>
-    <row r="40" spans="1:29" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:29" ht="15" customHeight="1">
       <c r="B40" s="614"/>
       <c r="C40" s="547" t="s">
         <v>649</v>
@@ -13582,7 +13576,7 @@
       <c r="P40" s="531"/>
       <c r="AB40" s="531"/>
     </row>
-    <row r="41" spans="1:29" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:29" ht="15" customHeight="1" thickBot="1">
       <c r="A41" s="527"/>
       <c r="B41" s="748"/>
       <c r="C41" s="565" t="s">
@@ -13614,7 +13608,7 @@
       <c r="AA41" s="531"/>
       <c r="AB41" s="531"/>
     </row>
-    <row r="42" spans="1:29" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:29" ht="15" customHeight="1">
       <c r="A42" s="531"/>
       <c r="B42" s="616"/>
       <c r="C42" s="549" t="s">
@@ -13644,7 +13638,7 @@
       <c r="AA42" s="531"/>
       <c r="AB42" s="531"/>
     </row>
-    <row r="43" spans="1:29" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:29" ht="15" customHeight="1">
       <c r="A43" s="531"/>
       <c r="B43" s="617"/>
       <c r="C43" s="547" t="s">
@@ -13677,7 +13671,7 @@
       <c r="AB43" s="531"/>
       <c r="AC43" s="531"/>
     </row>
-    <row r="44" spans="1:29" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:29" ht="15" customHeight="1" thickBot="1">
       <c r="A44" s="531"/>
       <c r="B44" s="618"/>
       <c r="C44" s="548" t="s">
@@ -13709,7 +13703,7 @@
       <c r="AA44" s="531"/>
       <c r="AB44" s="531"/>
     </row>
-    <row r="45" spans="1:29" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:29" ht="15" customHeight="1" thickBot="1">
       <c r="D45" s="542"/>
       <c r="E45" s="542"/>
       <c r="F45" s="542"/>
@@ -13734,7 +13728,7 @@
       <c r="AA45" s="531"/>
       <c r="AB45" s="531"/>
     </row>
-    <row r="46" spans="1:29" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:29" ht="13.5" thickBot="1">
       <c r="B46" s="1177" t="inlineStr">
         <is>
           <t>Direttore del corso: </t>
@@ -13766,7 +13760,7 @@
       <c r="AA46" s="531"/>
       <c r="AB46" s="531"/>
     </row>
-    <row r="47" spans="1:29" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:29" ht="13.5" thickBot="1">
       <c r="B47" s="476"/>
       <c r="C47" s="477"/>
       <c r="D47" s="477"/>
@@ -13792,7 +13786,7 @@
       <c r="AA47" s="531"/>
       <c r="AB47" s="531"/>
     </row>
-    <row r="48" spans="1:29" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:29" ht="13.5" thickBot="1">
       <c r="B48" s="1189" t="s">
         <v>38</v>
       </c>
@@ -13820,7 +13814,7 @@
       <c r="AA48" s="531"/>
       <c r="AB48" s="531"/>
     </row>
-    <row r="49" spans="2:16" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="49" spans="2:16" ht="13.5" thickBot="1">
       <c r="B49" s="535" t="s">
         <v>39</v>
       </c>
@@ -13845,7 +13839,7 @@
       <c r="O49" s="1220"/>
       <c r="P49" s="488"/>
     </row>
-    <row r="50" spans="2:16" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="50" spans="2:16" ht="14.1" customHeight="1">
       <c r="B50" s="552"/>
       <c r="C50" s="1223"/>
       <c r="D50" s="1224"/>
@@ -13862,7 +13856,7 @@
       <c r="O50" s="1224"/>
       <c r="P50" s="488"/>
     </row>
-    <row r="51" spans="2:16" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="51" spans="2:16" ht="14.1" customHeight="1">
       <c r="B51" s="532"/>
       <c r="C51" s="1215"/>
       <c r="D51" s="1216"/>
@@ -13878,7 +13872,7 @@
       <c r="N51" s="1216"/>
       <c r="O51" s="1217"/>
     </row>
-    <row r="52" spans="2:16" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="52" spans="2:16" ht="14.1" customHeight="1">
       <c r="B52" s="532"/>
       <c r="C52" s="1215"/>
       <c r="D52" s="1216"/>
@@ -13895,7 +13889,7 @@
       <c r="O52" s="1216"/>
       <c r="P52" s="488"/>
     </row>
-    <row r="53" spans="2:16" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="53" spans="2:16" ht="14.1" customHeight="1">
       <c r="B53" s="532"/>
       <c r="C53" s="1215"/>
       <c r="D53" s="1216"/>
@@ -13911,7 +13905,7 @@
       <c r="N53" s="1216"/>
       <c r="O53" s="1217"/>
     </row>
-    <row r="54" spans="2:16" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="54" spans="2:16" ht="14.1" customHeight="1">
       <c r="B54" s="532"/>
       <c r="C54" s="1215"/>
       <c r="D54" s="1216"/>
@@ -13928,7 +13922,7 @@
       <c r="O54" s="1216"/>
       <c r="P54" s="488"/>
     </row>
-    <row r="55" spans="2:16" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="55" spans="2:16" ht="14.1" customHeight="1">
       <c r="B55" s="532"/>
       <c r="C55" s="1215"/>
       <c r="D55" s="1216"/>
@@ -13944,7 +13938,7 @@
       <c r="O55" s="1216"/>
       <c r="P55" s="488"/>
     </row>
-    <row r="56" spans="2:16" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="56" spans="2:16" ht="14.1" customHeight="1">
       <c r="B56" s="532"/>
       <c r="C56" s="1215"/>
       <c r="D56" s="1216"/>
@@ -13961,7 +13955,7 @@
       <c r="O56" s="1216"/>
       <c r="P56" s="488"/>
     </row>
-    <row r="57" spans="2:16" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="57" spans="2:16" ht="14.1" customHeight="1">
       <c r="B57" s="532"/>
       <c r="C57" s="1215"/>
       <c r="D57" s="1216"/>
@@ -13978,7 +13972,7 @@
       <c r="O57" s="1216"/>
       <c r="P57" s="488"/>
     </row>
-    <row r="58" spans="2:16" ht="14.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="58" spans="2:16" ht="14.1" customHeight="1" thickBot="1">
       <c r="B58" s="553"/>
       <c r="C58" s="1240"/>
       <c r="D58" s="1241"/>
@@ -13994,7 +13988,7 @@
       <c r="N58" s="1241"/>
       <c r="O58" s="1242"/>
     </row>
-    <row r="59" spans="2:16" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="59" spans="2:16" ht="14.1" customHeight="1">
       <c r="B59" s="536"/>
       <c r="C59" s="1239"/>
       <c r="D59" s="1239"/>
@@ -14003,7 +13997,7 @@
       <c r="H59" s="534"/>
       <c r="I59" s="528"/>
     </row>
-    <row r="60" spans="2:16" ht="14.45" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="60" spans="2:16" ht="14.45" customHeight="1">
       <c r="C60" s="537"/>
       <c r="D60" s="537"/>
       <c r="E60" s="537"/>
@@ -14018,7 +14012,7 @@
       <c r="N60" s="534"/>
       <c r="O60" s="534"/>
     </row>
-    <row r="62" spans="2:16" x14ac:dyDescent="0.2">
+    <row r="62" spans="2:16">
       <c r="I62" s="1229"/>
       <c r="J62" s="1229"/>
       <c r="K62" s="1229"/>
@@ -14026,7 +14020,7 @@
       <c r="M62" s="1229"/>
       <c r="N62" s="1229"/>
     </row>
-    <row r="63" spans="2:16" x14ac:dyDescent="0.2">
+    <row r="63" spans="2:16">
       <c r="I63" s="1229"/>
       <c r="J63" s="1229"/>
       <c r="K63" s="1229"/>
@@ -14034,7 +14028,7 @@
       <c r="M63" s="1229"/>
       <c r="N63" s="1229"/>
     </row>
-    <row r="64" spans="2:16" x14ac:dyDescent="0.2">
+    <row r="64" spans="2:16">
       <c r="I64" s="1229"/>
       <c r="J64" s="1229"/>
       <c r="K64" s="1229"/>
@@ -14042,7 +14036,7 @@
       <c r="M64" s="1229"/>
       <c r="N64" s="1229"/>
     </row>
-    <row r="65" spans="9:14" x14ac:dyDescent="0.2">
+    <row r="65" spans="9:14">
       <c r="I65" s="529"/>
       <c r="J65" s="529"/>
       <c r="K65" s="530"/>
@@ -14257,8 +14251,7 @@
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.25" right="0.25" top="0.3" bottom="0.3" header="0.2" footer="0.2"/>
-  <!-- corsi-print -->
-  <pageSetup paperSize="9" fitToWidth="1" fitToHeight="1" orientation="landscape" r:id="rId1"/>
+  <pageSetup paperSize="9" fitToWidth="1" fitToHeight="1" orientation="landscape"/>
   <colBreaks count="1" manualBreakCount="1">
     <brk id="16" max="1048575" man="1"/>
   </colBreaks>

</xml_diff>

<commit_message>
fix(excel): truncate long PS module titles, re-clear blank
Keep official 66_PS EI layout; leave aula/TASK empty when unknown; fit addestramento to 42 chars for print.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/assets/templates/ps_weekly_blank.xlsx
+++ b/assets/templates/ps_weekly_blank.xlsx
@@ -4,6 +4,9 @@
   <sheets>
     <sheet name="Settimana" sheetId="1" r:id="rId1"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Settimana'!$A$1:$O$70</definedName>
+  </definedNames>
 </workbook>
 </file>
 
@@ -10427,6 +10430,7 @@
     <xf numFmtId="1" fontId="71" fillId="0" borderId="4" xfId="29" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
     </xf>
+    <!-- corsi-module-xfs -->
     <xf numFmtId="0" fontId="109" fillId="82" borderId="137" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
     </xf>

</xml_diff>

<commit_message>
fix(excel): paint full PS merges and restore official column alignment
Bad export (6) left E/F/J uncolored and forced left align on hour columns; reinject left/center module xfs, ASCII truncation, clean LOCALITA header.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/assets/templates/ps_weekly_blank.xlsx
+++ b/assets/templates/ps_weekly_blank.xlsx
@@ -2331,7 +2331,7 @@
     <numFmt numFmtId="171" formatCode="#,##0_ ;[Red]\-#,##0\ "/>
     <numFmt numFmtId="172" formatCode="[$-F800]dddd\,\ mmmm\ dd\,\ yyyy"/>
   </numFmts>
-  <fonts count="110" x14ac:knownFonts="1">
+  <fonts count="112" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -3032,6 +3032,22 @@
       <name val="Arial"/>
       <family val="2"/>
     </font>
+    <font>
+      <!-- corsi-white -->
+      <b/>
+      <sz val="9"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <!-- corsi-dark -->
+      <b/>
+      <sz val="9"/>
+      <color rgb="FF111827"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="102">
     <fill>
@@ -6315,7 +6331,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1313">
+  <cellXfs count="1333">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="66" fillId="0" borderId="0" xfId="29" applyFont="1"/>
     <xf numFmtId="0" fontId="78" fillId="0" borderId="0" xfId="29" applyFont="1"/>
@@ -10431,65 +10447,125 @@
       <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
     </xf>
     <!-- corsi-module-xfs -->
-    <xf numFmtId="0" fontId="109" fillId="82" borderId="137" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="109" fillId="83" borderId="137" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="109" fillId="84" borderId="137" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="109" fillId="85" borderId="137" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="109" fillId="86" borderId="137" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="109" fillId="87" borderId="137" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="109" fillId="88" borderId="137" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="109" fillId="89" borderId="137" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="109" fillId="90" borderId="137" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="109" fillId="91" borderId="137" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="109" fillId="92" borderId="137" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="109" fillId="93" borderId="137" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="109" fillId="94" borderId="137" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="109" fillId="95" borderId="137" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="109" fillId="96" borderId="137" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="108" fillId="97" borderId="137" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="108" fillId="98" borderId="137" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="108" fillId="99" borderId="137" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="108" fillId="100" borderId="137" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="108" fillId="101" borderId="137" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
+    <xf numFmtId="0" fontId="110" fillId="82" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="110" fillId="82" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="110" fillId="83" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="110" fillId="83" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="111" fillId="84" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="111" fillId="84" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="111" fillId="85" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="111" fillId="85" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="111" fillId="86" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="111" fillId="86" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="111" fillId="87" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="111" fillId="87" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="111" fillId="88" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="111" fillId="88" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="110" fillId="89" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="110" fillId="89" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="110" fillId="90" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="110" fillId="90" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="110" fillId="91" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="110" fillId="91" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="110" fillId="92" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="110" fillId="92" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="110" fillId="93" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="110" fillId="93" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="110" fillId="94" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="110" fillId="94" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="111" fillId="95" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="111" fillId="95" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="110" fillId="96" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="110" fillId="96" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="110" fillId="97" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="110" fillId="97" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="110" fillId="98" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="110" fillId="98" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="110" fillId="99" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="110" fillId="99" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="110" fillId="100" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="110" fillId="100" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="110" fillId="101" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="110" fillId="101" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="971">
@@ -12752,8 +12828,10 @@
       </c>
       <c r="L8" s="1270"/>
       <c r="M8" s="1271"/>
-      <c r="N8" s="1281" t="s">
-        <v>678</v>
+      <c r="N8" s="1281" t="inlineStr">
+        <is>
+          <t>LOCALITA'</t>
+        </is>
       </c>
       <c r="O8" s="1282"/>
       <c r="Q8" s="531"/>

</xml_diff>

<commit_message>
fix(excel): map PS lessons past Disposizione and lunch, black module text
Skip first-hour Disposizione and yellow pausa rows when filling; re-derive blank from Desktop 66_PS and force black text on module fills.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/assets/templates/ps_weekly_blank.xlsx
+++ b/assets/templates/ps_weekly_blank.xlsx
@@ -2331,7 +2331,7 @@
     <numFmt numFmtId="171" formatCode="#,##0_ ;[Red]\-#,##0\ "/>
     <numFmt numFmtId="172" formatCode="[$-F800]dddd\,\ mmmm\ dd\,\ yyyy"/>
   </numFmts>
-  <fonts count="112" x14ac:knownFonts="1">
+  <fonts count="109" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -3019,32 +3019,10 @@
       <family val="2"/>
     </font>
     <font>
-      <b/>
-      <sz val="8"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="Arial"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="8"/>
-      <color rgb="FF111827"/>
-      <name val="Arial"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <!-- corsi-white -->
-      <b/>
-      <sz val="9"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="Arial"/>
-      <family val="2"/>
-    </font>
-    <font>
       <!-- corsi-dark -->
       <b/>
       <sz val="9"/>
-      <color rgb="FF111827"/>
+      <color rgb="FF000000"/>
       <name val="Arial"/>
       <family val="2"/>
     </font>
@@ -3630,7 +3608,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="138">
+  <borders count="137">
     <border>
       <left/>
       <right/>
@@ -5342,21 +5320,6 @@
         <color indexed="64"/>
       </diagonal>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="971">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -10447,124 +10410,124 @@
       <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
     </xf>
     <!-- corsi-module-xfs -->
-    <xf numFmtId="0" fontId="110" fillId="82" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="110" fillId="82" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="110" fillId="83" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="110" fillId="83" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="111" fillId="84" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="111" fillId="84" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="111" fillId="85" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="111" fillId="85" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="111" fillId="86" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="111" fillId="86" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="111" fillId="87" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="111" fillId="87" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="111" fillId="88" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="111" fillId="88" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="110" fillId="89" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="110" fillId="89" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="110" fillId="90" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="110" fillId="90" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="110" fillId="91" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="110" fillId="91" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="110" fillId="92" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="110" fillId="92" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="110" fillId="93" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="110" fillId="93" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="110" fillId="94" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="110" fillId="94" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="111" fillId="95" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="111" fillId="95" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="110" fillId="96" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="110" fillId="96" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="110" fillId="97" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="110" fillId="97" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="110" fillId="98" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="110" fillId="98" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="110" fillId="99" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="110" fillId="99" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="110" fillId="100" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="110" fillId="100" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="110" fillId="101" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="110" fillId="101" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="108" fillId="82" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="108" fillId="82" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="108" fillId="83" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="108" fillId="83" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="108" fillId="84" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="108" fillId="84" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="108" fillId="85" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="108" fillId="85" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="108" fillId="86" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="108" fillId="86" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="108" fillId="87" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="108" fillId="87" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="108" fillId="88" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="108" fillId="88" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="108" fillId="89" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="108" fillId="89" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="108" fillId="90" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="108" fillId="90" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="108" fillId="91" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="108" fillId="91" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="108" fillId="92" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="108" fillId="92" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="108" fillId="93" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="108" fillId="93" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="108" fillId="94" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="108" fillId="94" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="108" fillId="95" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="108" fillId="95" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="108" fillId="96" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="108" fillId="96" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="108" fillId="97" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="108" fillId="97" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="108" fillId="98" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="108" fillId="98" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="108" fillId="99" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="108" fillId="99" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="108" fillId="100" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="108" fillId="100" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="108" fillId="101" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="108" fillId="101" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
     </xf>
   </cellXfs>
@@ -12655,13 +12618,13 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{368E55A2-AD71-4714-92B2-F8C5DEE7E7F4}">
   <sheetPr>
     <tabColor rgb="FF00B0F0"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:O70"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="12.75"/>
+  <dimension ref="A1:AG65"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="3" style="421" customWidth="1"/>
     <col min="2" max="2" width="11" style="421" bestFit="1" customWidth="1"/>
@@ -12679,12 +12642,12 @@
     <col min="17" max="16384" width="9.140625" style="421"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:33" ht="15" customHeight="1" thickBot="1">
+    <row r="1" spans="1:33" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A1" s="421" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:33" ht="15" customHeight="1">
+    <row r="2" spans="1:33" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B2" s="1258" t="s">
         <v>0</v>
       </c>
@@ -12705,7 +12668,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:33" ht="15" customHeight="1">
+    <row r="3" spans="1:33" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B3" s="1261" t="s">
         <v>9</v>
       </c>
@@ -12723,7 +12686,7 @@
       <c r="N3" s="1262"/>
       <c r="O3" s="1263"/>
     </row>
-    <row r="4" spans="1:33" ht="15" customHeight="1">
+    <row r="4" spans="1:33" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B4" s="1261" t="s">
         <v>652</v>
       </c>
@@ -12741,7 +12704,7 @@
       <c r="N4" s="1262"/>
       <c r="O4" s="1263"/>
     </row>
-    <row r="5" spans="1:33" ht="15" customHeight="1" thickBot="1">
+    <row r="5" spans="1:33" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B5" s="1264" t="inlineStr">
         <is>
           <t>{{COURSE_TITLE}}</t>
@@ -12761,7 +12724,7 @@
       <c r="N5" s="1265"/>
       <c r="O5" s="1266"/>
     </row>
-    <row r="6" spans="1:33" ht="15" customHeight="1" thickBot="1">
+    <row r="6" spans="1:33" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B6" s="683" t="s">
         <v>11</v>
       </c>
@@ -12781,7 +12744,7 @@
       <c r="N6" s="1070"/>
       <c r="O6" s="1071"/>
     </row>
-    <row r="7" spans="1:33" ht="15" customHeight="1" thickBot="1">
+    <row r="7" spans="1:33" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B7" s="690" t="s">
         <v>1</v>
       </c>
@@ -12801,7 +12764,7 @@
       <c r="N7" s="1073"/>
       <c r="O7" s="1074"/>
     </row>
-    <row r="8" spans="1:33" ht="15" customHeight="1">
+    <row r="8" spans="1:33" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B8" s="699" t="s">
         <v>2</v>
       </c>
@@ -12852,7 +12815,7 @@
       <c r="AF8" s="531"/>
       <c r="AG8" s="531"/>
     </row>
-    <row r="9" spans="1:33" ht="15" customHeight="1" thickBot="1">
+    <row r="9" spans="1:33" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B9" s="700"/>
       <c r="C9" s="702"/>
       <c r="D9" s="703"/>
@@ -12878,12 +12841,14 @@
       <c r="AF9" s="531"/>
       <c r="AG9" s="531"/>
     </row>
-    <row r="10" spans="1:33" ht="15" customHeight="1">
+    <row r="10" spans="1:33" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B10" s="613"/>
       <c r="C10" s="539" t="s">
         <v>67</v>
       </c>
-      <c r="D10" s="1159"/>
+      <c r="D10" s="1159" t="s">
+        <v>141</v>
+      </c>
       <c r="E10" s="1159"/>
       <c r="F10" s="1159"/>
       <c r="G10" s="541"/>
@@ -12902,7 +12867,7 @@
       <c r="AF10" s="531"/>
       <c r="AG10" s="531"/>
     </row>
-    <row r="11" spans="1:33" ht="15" customHeight="1">
+    <row r="11" spans="1:33" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B11" s="614"/>
       <c r="C11" s="547" t="s">
         <v>643</v>
@@ -12937,7 +12902,7 @@
       <c r="AF11" s="531"/>
       <c r="AG11" s="531"/>
     </row>
-    <row r="12" spans="1:33" ht="15" customHeight="1">
+    <row r="12" spans="1:33" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B12" s="614"/>
       <c r="C12" s="547" t="s">
         <v>644</v>
@@ -12970,7 +12935,7 @@
       <c r="AF12" s="531"/>
       <c r="AG12" s="531"/>
     </row>
-    <row r="13" spans="1:33" ht="15" customHeight="1">
+    <row r="13" spans="1:33" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B13" s="614"/>
       <c r="C13" s="547" t="s">
         <v>645</v>
@@ -13004,7 +12969,7 @@
       <c r="AF13" s="531"/>
       <c r="AG13" s="531"/>
     </row>
-    <row r="14" spans="1:33" ht="15" customHeight="1">
+    <row r="14" spans="1:33" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B14" s="614"/>
       <c r="C14" s="547" t="s">
         <v>670</v>
@@ -13025,7 +12990,7 @@
       <c r="AA14" s="531"/>
       <c r="AB14" s="531"/>
     </row>
-    <row r="15" spans="1:33" ht="15" customHeight="1">
+    <row r="15" spans="1:33" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B15" s="614"/>
       <c r="C15" s="540" t="s">
         <v>671</v>
@@ -13040,7 +13005,7 @@
       <c r="K15" s="567"/>
       <c r="L15" s="568"/>
       <c r="M15" s="567"/>
-      <c r="N15" s="1230"/>
+      <c r="N15" s="1278"/>
       <c r="O15" s="1231"/>
       <c r="AA15" s="531"/>
       <c r="AB15" s="531"/>
@@ -13050,7 +13015,7 @@
       <c r="AF15" s="531"/>
       <c r="AG15" s="531"/>
     </row>
-    <row r="16" spans="1:33" ht="15" customHeight="1">
+    <row r="16" spans="1:33" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B16" s="614"/>
       <c r="C16" s="547" t="s">
         <v>649</v>
@@ -13075,7 +13040,7 @@
       <c r="AF16" s="531"/>
       <c r="AG16" s="531"/>
     </row>
-    <row r="17" spans="2:33" ht="15" customHeight="1" thickBot="1">
+    <row r="17" spans="2:33" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B17" s="615"/>
       <c r="C17" s="548" t="s">
         <v>74</v>
@@ -13101,12 +13066,14 @@
       <c r="AF17" s="531"/>
       <c r="AG17" s="531"/>
     </row>
-    <row r="18" spans="2:33" ht="15" customHeight="1">
+    <row r="18" spans="2:33" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B18" s="613"/>
       <c r="C18" s="549" t="s">
         <v>67</v>
       </c>
-      <c r="D18" s="1159"/>
+      <c r="D18" s="1159" t="s">
+        <v>141</v>
+      </c>
       <c r="E18" s="1159"/>
       <c r="F18" s="1159"/>
       <c r="G18" s="541"/>
@@ -13125,7 +13092,7 @@
       <c r="AF18" s="531"/>
       <c r="AG18" s="531"/>
     </row>
-    <row r="19" spans="2:33" ht="15" customHeight="1">
+    <row r="19" spans="2:33" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B19" s="614"/>
       <c r="C19" s="547" t="s">
         <v>643</v>
@@ -13150,7 +13117,7 @@
       <c r="AF19" s="531"/>
       <c r="AG19" s="531"/>
     </row>
-    <row r="20" spans="2:33" ht="15" customHeight="1">
+    <row r="20" spans="2:33" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B20" s="614"/>
       <c r="C20" s="547" t="s">
         <v>644</v>
@@ -13171,7 +13138,7 @@
       <c r="AB20" s="531"/>
       <c r="AC20" s="531"/>
     </row>
-    <row r="21" spans="2:33" ht="15" customHeight="1">
+    <row r="21" spans="2:33" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B21" s="614"/>
       <c r="C21" s="547" t="s">
         <v>645</v>
@@ -13192,7 +13159,7 @@
       <c r="AB21" s="531"/>
       <c r="AC21" s="531"/>
     </row>
-    <row r="22" spans="2:33" ht="15" customHeight="1">
+    <row r="22" spans="2:33" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B22" s="614"/>
       <c r="C22" s="547" t="s">
         <v>670</v>
@@ -13214,7 +13181,7 @@
       <c r="AB22" s="531"/>
       <c r="AC22" s="531"/>
     </row>
-    <row r="23" spans="2:33" ht="15" customHeight="1">
+    <row r="23" spans="2:33" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B23" s="614"/>
       <c r="C23" s="550" t="s">
         <v>671</v>
@@ -13229,7 +13196,7 @@
       <c r="K23" s="558"/>
       <c r="L23" s="558"/>
       <c r="M23" s="558"/>
-      <c r="N23" s="1230"/>
+      <c r="N23" s="1278"/>
       <c r="O23" s="1231"/>
       <c r="S23" s="531"/>
       <c r="T23" s="531"/>
@@ -13242,7 +13209,7 @@
       <c r="AA23" s="531"/>
       <c r="AB23" s="531"/>
     </row>
-    <row r="24" spans="2:33" ht="15" customHeight="1">
+    <row r="24" spans="2:33" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B24" s="614"/>
       <c r="C24" s="547" t="s">
         <v>649</v>
@@ -13270,7 +13237,7 @@
       <c r="AA24" s="531"/>
       <c r="AB24" s="531"/>
     </row>
-    <row r="25" spans="2:33" ht="15" customHeight="1" thickBot="1">
+    <row r="25" spans="2:33" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B25" s="615"/>
       <c r="C25" s="548" t="s">
         <v>74</v>
@@ -13290,12 +13257,14 @@
       <c r="P25" s="531"/>
       <c r="S25" s="531"/>
     </row>
-    <row r="26" spans="2:33" ht="15" customHeight="1">
+    <row r="26" spans="2:33" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B26" s="613"/>
       <c r="C26" s="549" t="s">
         <v>67</v>
       </c>
-      <c r="D26" s="1159"/>
+      <c r="D26" s="1159" t="s">
+        <v>141</v>
+      </c>
       <c r="E26" s="1159"/>
       <c r="F26" s="1159"/>
       <c r="G26" s="541"/>
@@ -13319,7 +13288,7 @@
       <c r="AA26" s="531"/>
       <c r="AB26" s="531"/>
     </row>
-    <row r="27" spans="2:33" ht="15" customHeight="1">
+    <row r="27" spans="2:33" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B27" s="614"/>
       <c r="C27" s="554" t="s">
         <v>643</v>
@@ -13338,7 +13307,7 @@
       <c r="O27" s="1231"/>
       <c r="Q27" s="531"/>
     </row>
-    <row r="28" spans="2:33" ht="15" customHeight="1">
+    <row r="28" spans="2:33" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B28" s="614"/>
       <c r="C28" s="554" t="s">
         <v>644</v>
@@ -13358,7 +13327,7 @@
       <c r="P28" s="531"/>
       <c r="Q28" s="531"/>
     </row>
-    <row r="29" spans="2:33" ht="15" customHeight="1">
+    <row r="29" spans="2:33" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B29" s="614"/>
       <c r="C29" s="554" t="s">
         <v>645</v>
@@ -13387,7 +13356,7 @@
       <c r="AA29" s="531"/>
       <c r="AB29" s="531"/>
     </row>
-    <row r="30" spans="2:33" ht="15" customHeight="1">
+    <row r="30" spans="2:33" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B30" s="614"/>
       <c r="C30" s="554" t="s">
         <v>670</v>
@@ -13407,7 +13376,7 @@
       <c r="P30" s="531"/>
       <c r="S30" s="531"/>
     </row>
-    <row r="31" spans="2:33" ht="15" customHeight="1">
+    <row r="31" spans="2:33" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B31" s="614"/>
       <c r="C31" s="583" t="s">
         <v>671</v>
@@ -13422,12 +13391,12 @@
       <c r="K31" s="576"/>
       <c r="L31" s="576"/>
       <c r="M31" s="576"/>
-      <c r="N31" s="1249"/>
+      <c r="N31" s="1278"/>
       <c r="O31" s="1231"/>
       <c r="Q31" s="531"/>
       <c r="S31" s="531"/>
     </row>
-    <row r="32" spans="2:33" ht="15" customHeight="1">
+    <row r="32" spans="2:33" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B32" s="614"/>
       <c r="C32" s="554" t="s">
         <v>649</v>
@@ -13447,7 +13416,7 @@
       <c r="Q32" s="531"/>
       <c r="AB32" s="531"/>
     </row>
-    <row r="33" spans="1:29" ht="15" customHeight="1" thickBot="1">
+    <row r="33" spans="1:29" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B33" s="615"/>
       <c r="C33" s="561" t="s">
         <v>74</v>
@@ -13468,12 +13437,14 @@
       <c r="Q33" s="531"/>
       <c r="AB33" s="531"/>
     </row>
-    <row r="34" spans="1:29" ht="15" customHeight="1">
+    <row r="34" spans="1:29" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B34" s="613"/>
       <c r="C34" s="549" t="s">
         <v>67</v>
       </c>
-      <c r="D34" s="1159"/>
+      <c r="D34" s="1159" t="s">
+        <v>141</v>
+      </c>
       <c r="E34" s="1159"/>
       <c r="F34" s="1159"/>
       <c r="G34" s="541"/>
@@ -13498,7 +13469,7 @@
       <c r="AA34" s="531"/>
       <c r="AB34" s="531"/>
     </row>
-    <row r="35" spans="1:29" ht="15" customHeight="1">
+    <row r="35" spans="1:29" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B35" s="614"/>
       <c r="C35" s="547" t="s">
         <v>643</v>
@@ -13528,7 +13499,7 @@
       <c r="AA35" s="531"/>
       <c r="AB35" s="531"/>
     </row>
-    <row r="36" spans="1:29" ht="15" customHeight="1">
+    <row r="36" spans="1:29" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B36" s="614"/>
       <c r="C36" s="547" t="s">
         <v>644</v>
@@ -13559,7 +13530,7 @@
       <c r="AA36" s="531"/>
       <c r="AB36" s="531"/>
     </row>
-    <row r="37" spans="1:29" ht="15" customHeight="1">
+    <row r="37" spans="1:29" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B37" s="614"/>
       <c r="C37" s="547" t="s">
         <v>645</v>
@@ -13589,7 +13560,7 @@
       <c r="AA37" s="531"/>
       <c r="AB37" s="531"/>
     </row>
-    <row r="38" spans="1:29" ht="15" customHeight="1">
+    <row r="38" spans="1:29" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B38" s="614"/>
       <c r="C38" s="554" t="s">
         <v>670</v>
@@ -13619,7 +13590,7 @@
       <c r="AA38" s="531"/>
       <c r="AB38" s="531"/>
     </row>
-    <row r="39" spans="1:29" ht="15" customHeight="1">
+    <row r="39" spans="1:29" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B39" s="614"/>
       <c r="C39" s="550" t="s">
         <v>671</v>
@@ -13634,11 +13605,11 @@
       <c r="K39" s="578"/>
       <c r="L39" s="566"/>
       <c r="M39" s="566"/>
-      <c r="N39" s="1230"/>
+      <c r="N39" s="1278"/>
       <c r="O39" s="1231"/>
       <c r="AB39" s="531"/>
     </row>
-    <row r="40" spans="1:29" ht="15" customHeight="1">
+    <row r="40" spans="1:29" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B40" s="614"/>
       <c r="C40" s="547" t="s">
         <v>649</v>
@@ -13658,7 +13629,7 @@
       <c r="P40" s="531"/>
       <c r="AB40" s="531"/>
     </row>
-    <row r="41" spans="1:29" ht="15" customHeight="1" thickBot="1">
+    <row r="41" spans="1:29" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A41" s="527"/>
       <c r="B41" s="748"/>
       <c r="C41" s="565" t="s">
@@ -13690,7 +13661,7 @@
       <c r="AA41" s="531"/>
       <c r="AB41" s="531"/>
     </row>
-    <row r="42" spans="1:29" ht="15" customHeight="1">
+    <row r="42" spans="1:29" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A42" s="531"/>
       <c r="B42" s="616"/>
       <c r="C42" s="549" t="s">
@@ -13720,7 +13691,7 @@
       <c r="AA42" s="531"/>
       <c r="AB42" s="531"/>
     </row>
-    <row r="43" spans="1:29" ht="15" customHeight="1">
+    <row r="43" spans="1:29" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A43" s="531"/>
       <c r="B43" s="617"/>
       <c r="C43" s="547" t="s">
@@ -13753,7 +13724,7 @@
       <c r="AB43" s="531"/>
       <c r="AC43" s="531"/>
     </row>
-    <row r="44" spans="1:29" ht="15" customHeight="1" thickBot="1">
+    <row r="44" spans="1:29" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A44" s="531"/>
       <c r="B44" s="618"/>
       <c r="C44" s="548" t="s">
@@ -13785,7 +13756,7 @@
       <c r="AA44" s="531"/>
       <c r="AB44" s="531"/>
     </row>
-    <row r="45" spans="1:29" ht="15" customHeight="1" thickBot="1">
+    <row r="45" spans="1:29" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="D45" s="542"/>
       <c r="E45" s="542"/>
       <c r="F45" s="542"/>
@@ -13810,7 +13781,7 @@
       <c r="AA45" s="531"/>
       <c r="AB45" s="531"/>
     </row>
-    <row r="46" spans="1:29" ht="13.5" thickBot="1">
+    <row r="46" spans="1:29" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B46" s="1177" t="inlineStr">
         <is>
           <t>Direttore del corso: </t>
@@ -13842,7 +13813,7 @@
       <c r="AA46" s="531"/>
       <c r="AB46" s="531"/>
     </row>
-    <row r="47" spans="1:29" ht="13.5" thickBot="1">
+    <row r="47" spans="1:29" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B47" s="476"/>
       <c r="C47" s="477"/>
       <c r="D47" s="477"/>
@@ -13868,7 +13839,7 @@
       <c r="AA47" s="531"/>
       <c r="AB47" s="531"/>
     </row>
-    <row r="48" spans="1:29" ht="13.5" thickBot="1">
+    <row r="48" spans="1:29" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B48" s="1189" t="s">
         <v>38</v>
       </c>
@@ -13896,7 +13867,7 @@
       <c r="AA48" s="531"/>
       <c r="AB48" s="531"/>
     </row>
-    <row r="49" spans="2:16" ht="13.5" thickBot="1">
+    <row r="49" spans="2:16" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B49" s="535" t="s">
         <v>39</v>
       </c>
@@ -13921,7 +13892,7 @@
       <c r="O49" s="1220"/>
       <c r="P49" s="488"/>
     </row>
-    <row r="50" spans="2:16" ht="14.1" customHeight="1">
+    <row r="50" spans="2:16" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B50" s="552"/>
       <c r="C50" s="1223"/>
       <c r="D50" s="1224"/>
@@ -13938,7 +13909,7 @@
       <c r="O50" s="1224"/>
       <c r="P50" s="488"/>
     </row>
-    <row r="51" spans="2:16" ht="14.1" customHeight="1">
+    <row r="51" spans="2:16" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B51" s="532"/>
       <c r="C51" s="1215"/>
       <c r="D51" s="1216"/>
@@ -13954,7 +13925,7 @@
       <c r="N51" s="1216"/>
       <c r="O51" s="1217"/>
     </row>
-    <row r="52" spans="2:16" ht="14.1" customHeight="1">
+    <row r="52" spans="2:16" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B52" s="532"/>
       <c r="C52" s="1215"/>
       <c r="D52" s="1216"/>
@@ -13971,7 +13942,7 @@
       <c r="O52" s="1216"/>
       <c r="P52" s="488"/>
     </row>
-    <row r="53" spans="2:16" ht="14.1" customHeight="1">
+    <row r="53" spans="2:16" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B53" s="532"/>
       <c r="C53" s="1215"/>
       <c r="D53" s="1216"/>
@@ -13987,7 +13958,7 @@
       <c r="N53" s="1216"/>
       <c r="O53" s="1217"/>
     </row>
-    <row r="54" spans="2:16" ht="14.1" customHeight="1">
+    <row r="54" spans="2:16" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B54" s="532"/>
       <c r="C54" s="1215"/>
       <c r="D54" s="1216"/>
@@ -14004,7 +13975,7 @@
       <c r="O54" s="1216"/>
       <c r="P54" s="488"/>
     </row>
-    <row r="55" spans="2:16" ht="14.1" customHeight="1">
+    <row r="55" spans="2:16" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B55" s="532"/>
       <c r="C55" s="1215"/>
       <c r="D55" s="1216"/>
@@ -14020,7 +13991,7 @@
       <c r="O55" s="1216"/>
       <c r="P55" s="488"/>
     </row>
-    <row r="56" spans="2:16" ht="14.1" customHeight="1">
+    <row r="56" spans="2:16" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B56" s="532"/>
       <c r="C56" s="1215"/>
       <c r="D56" s="1216"/>
@@ -14037,7 +14008,7 @@
       <c r="O56" s="1216"/>
       <c r="P56" s="488"/>
     </row>
-    <row r="57" spans="2:16" ht="14.1" customHeight="1">
+    <row r="57" spans="2:16" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B57" s="532"/>
       <c r="C57" s="1215"/>
       <c r="D57" s="1216"/>
@@ -14054,7 +14025,7 @@
       <c r="O57" s="1216"/>
       <c r="P57" s="488"/>
     </row>
-    <row r="58" spans="2:16" ht="14.1" customHeight="1" thickBot="1">
+    <row r="58" spans="2:16" ht="14.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B58" s="553"/>
       <c r="C58" s="1240"/>
       <c r="D58" s="1241"/>
@@ -14070,7 +14041,7 @@
       <c r="N58" s="1241"/>
       <c r="O58" s="1242"/>
     </row>
-    <row r="59" spans="2:16" ht="14.1" customHeight="1">
+    <row r="59" spans="2:16" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B59" s="536"/>
       <c r="C59" s="1239"/>
       <c r="D59" s="1239"/>
@@ -14079,7 +14050,7 @@
       <c r="H59" s="534"/>
       <c r="I59" s="528"/>
     </row>
-    <row r="60" spans="2:16" ht="14.45" customHeight="1">
+    <row r="60" spans="2:16" ht="14.45" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C60" s="537"/>
       <c r="D60" s="537"/>
       <c r="E60" s="537"/>
@@ -14094,7 +14065,7 @@
       <c r="N60" s="534"/>
       <c r="O60" s="534"/>
     </row>
-    <row r="62" spans="2:16">
+    <row r="62" spans="2:16" x14ac:dyDescent="0.2">
       <c r="I62" s="1229"/>
       <c r="J62" s="1229"/>
       <c r="K62" s="1229"/>
@@ -14102,7 +14073,7 @@
       <c r="M62" s="1229"/>
       <c r="N62" s="1229"/>
     </row>
-    <row r="63" spans="2:16">
+    <row r="63" spans="2:16" x14ac:dyDescent="0.2">
       <c r="I63" s="1229"/>
       <c r="J63" s="1229"/>
       <c r="K63" s="1229"/>
@@ -14110,7 +14081,7 @@
       <c r="M63" s="1229"/>
       <c r="N63" s="1229"/>
     </row>
-    <row r="64" spans="2:16">
+    <row r="64" spans="2:16" x14ac:dyDescent="0.2">
       <c r="I64" s="1229"/>
       <c r="J64" s="1229"/>
       <c r="K64" s="1229"/>
@@ -14118,7 +14089,7 @@
       <c r="M64" s="1229"/>
       <c r="N64" s="1229"/>
     </row>
-    <row r="65" spans="9:14">
+    <row r="65" spans="9:14" x14ac:dyDescent="0.2">
       <c r="I65" s="529"/>
       <c r="J65" s="529"/>
       <c r="K65" s="530"/>
@@ -14332,8 +14303,8 @@
       <formula>FLOOR(B34,1)=TODAY()</formula>
     </cfRule>
   </conditionalFormatting>
-  <pageMargins left="0.25" right="0.25" top="0.3" bottom="0.3" header="0.2" footer="0.2"/>
-  <pageSetup paperSize="9" fitToWidth="1" fitToHeight="1" orientation="landscape"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" fitToWidth="1" fitToHeight="1" orientation="landscape" r:id="rId1"/>
   <colBreaks count="1" manualBreakCount="1">
     <brk id="16" max="1048575" man="1"/>
   </colBreaks>

</xml_diff>

<commit_message>
fix(excel): restore PS LOCALITA/AULA header and EI/CC attendee columns
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/assets/templates/ps_weekly_blank.xlsx
+++ b/assets/templates/ps_weekly_blank.xlsx
@@ -12791,10 +12791,8 @@
       </c>
       <c r="L8" s="1270"/>
       <c r="M8" s="1271"/>
-      <c r="N8" s="1281" t="inlineStr">
-        <is>
-          <t>LOCALITA'</t>
-        </is>
+      <c r="N8" s="1281" t="s">
+        <v>678</v>
       </c>
       <c r="O8" s="1282"/>
       <c r="Q8" s="531"/>

</xml_diff>

<commit_message>
fix(excel): put CC attendees (LA RASPATA) on right; restore AM footer
forza=CC drives PERSONALE right column; blank keeps IL COMANDANTE / Accountable Manager from 66_PS.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/assets/templates/ps_weekly_blank.xlsx
+++ b/assets/templates/ps_weekly_blank.xlsx
@@ -14064,7 +14064,9 @@
       <c r="O60" s="534"/>
     </row>
     <row r="62" spans="2:16" x14ac:dyDescent="0.2">
-      <c r="I62" s="1229"/>
+      <c r="I62" s="1229" t="s">
+        <v>672</v>
+      </c>
       <c r="J62" s="1229"/>
       <c r="K62" s="1229"/>
       <c r="L62" s="1229"/>
@@ -14072,7 +14074,9 @@
       <c r="N62" s="1229"/>
     </row>
     <row r="63" spans="2:16" x14ac:dyDescent="0.2">
-      <c r="I63" s="1229"/>
+      <c r="I63" s="1229" t="s">
+        <v>673</v>
+      </c>
       <c r="J63" s="1229"/>
       <c r="K63" s="1229"/>
       <c r="L63" s="1229"/>

</xml_diff>

<commit_message>
feat(ps): aula 1-7, LOCALITA Excel e bordi N:O
Teoria esporta AULA n, pratica HANGAR 6; blank usa stile 1230 sulle lezioni (3 BTC default aula 3).

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/assets/templates/ps_weekly_blank.xlsx
+++ b/assets/templates/ps_weekly_blank.xlsx
@@ -12880,7 +12880,7 @@
       <c r="K11" s="560"/>
       <c r="L11" s="546"/>
       <c r="M11" s="541"/>
-      <c r="N11" s="1278"/>
+      <c r="N11" s="1230"/>
       <c r="O11" s="1231"/>
       <c r="Q11" s="531"/>
       <c r="R11" s="531"/>
@@ -12915,7 +12915,7 @@
       <c r="K12" s="560"/>
       <c r="L12" s="546"/>
       <c r="M12" s="541"/>
-      <c r="N12" s="1278"/>
+      <c r="N12" s="1230"/>
       <c r="O12" s="1231"/>
       <c r="Q12" s="531"/>
       <c r="R12" s="531"/>
@@ -12948,7 +12948,7 @@
       <c r="K13" s="560"/>
       <c r="L13" s="546"/>
       <c r="M13" s="541"/>
-      <c r="N13" s="1278"/>
+      <c r="N13" s="1230"/>
       <c r="O13" s="1231"/>
       <c r="P13" s="531"/>
       <c r="Q13" s="531"/>
@@ -12982,7 +12982,7 @@
       <c r="K14" s="560"/>
       <c r="L14" s="546"/>
       <c r="M14" s="541"/>
-      <c r="N14" s="1278"/>
+      <c r="N14" s="1230"/>
       <c r="O14" s="1231"/>
       <c r="P14" s="531"/>
       <c r="AA14" s="531"/>
@@ -13003,7 +13003,7 @@
       <c r="K15" s="567"/>
       <c r="L15" s="568"/>
       <c r="M15" s="567"/>
-      <c r="N15" s="1278"/>
+      <c r="N15" s="1230"/>
       <c r="O15" s="1231"/>
       <c r="AA15" s="531"/>
       <c r="AB15" s="531"/>
@@ -13028,7 +13028,7 @@
       <c r="K16" s="560"/>
       <c r="L16" s="546"/>
       <c r="M16" s="541"/>
-      <c r="N16" s="1278"/>
+      <c r="N16" s="1230"/>
       <c r="O16" s="1231"/>
       <c r="AA16" s="531"/>
       <c r="AB16" s="531"/>
@@ -13053,7 +13053,7 @@
       <c r="K17" s="560"/>
       <c r="L17" s="546"/>
       <c r="M17" s="541"/>
-      <c r="N17" s="1278"/>
+      <c r="N17" s="1230"/>
       <c r="O17" s="1253"/>
       <c r="P17" s="531"/>
       <c r="AA17" s="531"/>
@@ -13105,7 +13105,7 @@
       <c r="K19" s="560"/>
       <c r="L19" s="546"/>
       <c r="M19" s="541"/>
-      <c r="N19" s="1278"/>
+      <c r="N19" s="1230"/>
       <c r="O19" s="1231"/>
       <c r="P19" s="531"/>
       <c r="AB19" s="531"/>
@@ -13130,7 +13130,7 @@
       <c r="K20" s="560"/>
       <c r="L20" s="546"/>
       <c r="M20" s="541"/>
-      <c r="N20" s="1278"/>
+      <c r="N20" s="1230"/>
       <c r="O20" s="1231"/>
       <c r="P20" s="531"/>
       <c r="AB20" s="531"/>
@@ -13151,7 +13151,7 @@
       <c r="K21" s="560"/>
       <c r="L21" s="546"/>
       <c r="M21" s="541"/>
-      <c r="N21" s="1278"/>
+      <c r="N21" s="1230"/>
       <c r="O21" s="1231"/>
       <c r="P21" s="531"/>
       <c r="AB21" s="531"/>
@@ -13172,7 +13172,7 @@
       <c r="K22" s="560"/>
       <c r="L22" s="546"/>
       <c r="M22" s="541"/>
-      <c r="N22" s="1278"/>
+      <c r="N22" s="1230"/>
       <c r="O22" s="1231"/>
       <c r="P22" s="531"/>
       <c r="AA22" s="531"/>
@@ -13194,7 +13194,7 @@
       <c r="K23" s="558"/>
       <c r="L23" s="558"/>
       <c r="M23" s="558"/>
-      <c r="N23" s="1278"/>
+      <c r="N23" s="1230"/>
       <c r="O23" s="1231"/>
       <c r="S23" s="531"/>
       <c r="T23" s="531"/>
@@ -13222,7 +13222,7 @@
       <c r="K24" s="560"/>
       <c r="L24" s="546"/>
       <c r="M24" s="541"/>
-      <c r="N24" s="1278"/>
+      <c r="N24" s="1230"/>
       <c r="O24" s="1231"/>
       <c r="S24" s="531"/>
       <c r="T24" s="531"/>
@@ -13250,7 +13250,7 @@
       <c r="K25" s="560"/>
       <c r="L25" s="546"/>
       <c r="M25" s="541"/>
-      <c r="N25" s="1278"/>
+      <c r="N25" s="1230"/>
       <c r="O25" s="1231"/>
       <c r="P25" s="531"/>
       <c r="S25" s="531"/>
@@ -13301,7 +13301,7 @@
       <c r="K27" s="560"/>
       <c r="L27" s="546"/>
       <c r="M27" s="541"/>
-      <c r="N27" s="1278"/>
+      <c r="N27" s="1230"/>
       <c r="O27" s="1231"/>
       <c r="Q27" s="531"/>
     </row>
@@ -13320,7 +13320,7 @@
       <c r="K28" s="560"/>
       <c r="L28" s="546"/>
       <c r="M28" s="541"/>
-      <c r="N28" s="1278"/>
+      <c r="N28" s="1230"/>
       <c r="O28" s="1231"/>
       <c r="P28" s="531"/>
       <c r="Q28" s="531"/>
@@ -13340,7 +13340,7 @@
       <c r="K29" s="560"/>
       <c r="L29" s="546"/>
       <c r="M29" s="541"/>
-      <c r="N29" s="1278"/>
+      <c r="N29" s="1230"/>
       <c r="O29" s="1231"/>
       <c r="P29" s="531"/>
       <c r="S29" s="531"/>
@@ -13369,7 +13369,7 @@
       <c r="K30" s="560"/>
       <c r="L30" s="546"/>
       <c r="M30" s="541"/>
-      <c r="N30" s="1278"/>
+      <c r="N30" s="1230"/>
       <c r="O30" s="1231"/>
       <c r="P30" s="531"/>
       <c r="S30" s="531"/>
@@ -13389,7 +13389,7 @@
       <c r="K31" s="576"/>
       <c r="L31" s="576"/>
       <c r="M31" s="576"/>
-      <c r="N31" s="1278"/>
+      <c r="N31" s="1230"/>
       <c r="O31" s="1231"/>
       <c r="Q31" s="531"/>
       <c r="S31" s="531"/>
@@ -13409,7 +13409,7 @@
       <c r="K32" s="560"/>
       <c r="L32" s="546"/>
       <c r="M32" s="541"/>
-      <c r="N32" s="1278"/>
+      <c r="N32" s="1230"/>
       <c r="O32" s="1231"/>
       <c r="Q32" s="531"/>
       <c r="AB32" s="531"/>
@@ -13429,7 +13429,7 @@
       <c r="K33" s="560"/>
       <c r="L33" s="546"/>
       <c r="M33" s="541"/>
-      <c r="N33" s="1278"/>
+      <c r="N33" s="1230"/>
       <c r="O33" s="1253"/>
       <c r="P33" s="531"/>
       <c r="Q33" s="531"/>
@@ -13482,7 +13482,7 @@
       <c r="K35" s="560"/>
       <c r="L35" s="546"/>
       <c r="M35" s="541"/>
-      <c r="N35" s="1278"/>
+      <c r="N35" s="1230"/>
       <c r="O35" s="1231"/>
       <c r="Q35" s="531"/>
       <c r="R35" s="531"/>
@@ -13512,7 +13512,7 @@
       <c r="K36" s="560"/>
       <c r="L36" s="546"/>
       <c r="M36" s="541"/>
-      <c r="N36" s="1278"/>
+      <c r="N36" s="1230"/>
       <c r="O36" s="1231"/>
       <c r="P36" s="531"/>
       <c r="Q36" s="531"/>
@@ -13543,7 +13543,7 @@
       <c r="K37" s="560"/>
       <c r="L37" s="546"/>
       <c r="M37" s="541"/>
-      <c r="N37" s="1278"/>
+      <c r="N37" s="1230"/>
       <c r="O37" s="1231"/>
       <c r="P37" s="531"/>
       <c r="R37" s="531"/>
@@ -13573,7 +13573,7 @@
       <c r="K38" s="560"/>
       <c r="L38" s="546"/>
       <c r="M38" s="541"/>
-      <c r="N38" s="1278"/>
+      <c r="N38" s="1230"/>
       <c r="O38" s="1231"/>
       <c r="P38" s="531"/>
       <c r="R38" s="531"/>
@@ -13603,7 +13603,7 @@
       <c r="K39" s="578"/>
       <c r="L39" s="566"/>
       <c r="M39" s="566"/>
-      <c r="N39" s="1278"/>
+      <c r="N39" s="1230"/>
       <c r="O39" s="1231"/>
       <c r="AB39" s="531"/>
     </row>
@@ -13622,7 +13622,7 @@
       <c r="K40" s="560"/>
       <c r="L40" s="546"/>
       <c r="M40" s="541"/>
-      <c r="N40" s="1278"/>
+      <c r="N40" s="1230"/>
       <c r="O40" s="1231"/>
       <c r="P40" s="531"/>
       <c r="AB40" s="531"/>
@@ -13643,7 +13643,7 @@
       <c r="K41" s="560"/>
       <c r="L41" s="546"/>
       <c r="M41" s="541"/>
-      <c r="N41" s="1278"/>
+      <c r="N41" s="1230"/>
       <c r="O41" s="1233"/>
       <c r="P41" s="531"/>
       <c r="Q41" s="531"/>
@@ -13675,7 +13675,7 @@
       <c r="K42" s="560"/>
       <c r="L42" s="546"/>
       <c r="M42" s="541"/>
-      <c r="N42" s="1278"/>
+      <c r="N42" s="1230"/>
       <c r="O42" s="1247"/>
       <c r="R42" s="531"/>
       <c r="S42" s="531"/>
@@ -13705,7 +13705,7 @@
       <c r="K43" s="560"/>
       <c r="L43" s="546"/>
       <c r="M43" s="541"/>
-      <c r="N43" s="1278"/>
+      <c r="N43" s="1230"/>
       <c r="O43" s="1231"/>
       <c r="P43" s="531"/>
       <c r="Q43" s="531"/>
@@ -13738,7 +13738,7 @@
       <c r="K44" s="560"/>
       <c r="L44" s="546"/>
       <c r="M44" s="541"/>
-      <c r="N44" s="1278"/>
+      <c r="N44" s="1230"/>
       <c r="O44" s="1253"/>
       <c r="P44" s="531"/>
       <c r="Q44" s="531"/>

</xml_diff>

<commit_message>
fix(excel): stop PS print crash — drop printer DEVMODE, fit 1x1
Landscape fitToPage was paired with Desktop portrait printerSettings.bin and colBreaks, which crashed Excel Print Preview. Strip printer parts, breaks, and force single-page print area A1:O70.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/assets/templates/ps_weekly_blank.xlsx
+++ b/assets/templates/ps_weekly_blank.xlsx
@@ -1,12 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <workbookPr/>
+  <bookViews>
+    <workbookView windowWidth="20000" windowHeight="10000"/>
+  </bookViews>
   <sheets>
     <sheet name="Settimana" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'Settimana'!$A$1:$O$70</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">Settimana!$A$1:$O$70</definedName>
   </definedNames>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
@@ -14260,55 +14265,7 @@
     <mergeCell ref="N36:O36"/>
     <mergeCell ref="J55:O55"/>
   </mergeCells>
-  <conditionalFormatting sqref="B1">
-    <cfRule type="timePeriod" dxfId="8" priority="13" timePeriod="today">
-      <formula>FLOOR(B1,1)=TODAY()</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B69:B1048576">
-    <cfRule type="timePeriod" dxfId="7" priority="14" timePeriod="today">
-      <formula>FLOOR(B69,1)=TODAY()</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B2:B7">
-    <cfRule type="timePeriod" dxfId="6" priority="11" timePeriod="today">
-      <formula>FLOOR(B2,1)=TODAY()</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B46:B58 B61:B68">
-    <cfRule type="timePeriod" dxfId="5" priority="12" timePeriod="today">
-      <formula>FLOOR(B46,1)=TODAY()</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B8:B9">
-    <cfRule type="timePeriod" dxfId="4" priority="10" timePeriod="today">
-      <formula>FLOOR(B8,1)=TODAY()</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B42">
-    <cfRule type="timePeriod" dxfId="3" priority="4" timePeriod="today">
-      <formula>FLOOR(B42,1)=TODAY()</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B10 B26">
-    <cfRule type="timePeriod" dxfId="2" priority="3" timePeriod="today">
-      <formula>FLOOR(B10,1)=TODAY()</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B18">
-    <cfRule type="timePeriod" dxfId="1" priority="2" timePeriod="today">
-      <formula>FLOOR(B18,1)=TODAY()</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B34">
-    <cfRule type="timePeriod" dxfId="0" priority="1" timePeriod="today">
-      <formula>FLOOR(B34,1)=TODAY()</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" fitToWidth="1" fitToHeight="1" orientation="landscape" r:id="rId1"/>
-  <colBreaks count="1" manualBreakCount="1">
-    <brk id="16" max="1048575" man="1"/>
-  </colBreaks>
+  <pageMargins left="0.25" right="0.25" top="0.3" bottom="0.3" header="0.2" footer="0.2"/>
+  <pageSetup paperSize="9" fitToWidth="1" fitToHeight="1" orientation="landscape"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
fix(excel): PS print portrait + drop PDF settimana button
Portrait fit 1x1 with tighter margins; remove weekly PDF entry from director schedule UI (Excel PS unchanged).

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/assets/templates/ps_weekly_blank.xlsx
+++ b/assets/templates/ps_weekly_blank.xlsx
@@ -14265,7 +14265,7 @@
     <mergeCell ref="N36:O36"/>
     <mergeCell ref="J55:O55"/>
   </mergeCells>
-  <pageMargins left="0.25" right="0.25" top="0.3" bottom="0.3" header="0.2" footer="0.2"/>
-  <pageSetup paperSize="9" fitToWidth="1" fitToHeight="1" orientation="landscape"/>
+  <pageMargins left="0.2" right="0.2" top="0.25" bottom="0.25" header="0.15" footer="0.15"/>
+  <pageSetup paperSize="9" fitToWidth="1" fitToHeight="1" orientation="portrait"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
fix(planner): drag piu lento, lezioni validate/passate bloccate, Excel PS con colori tenui
- Drag: dwell 500 ms prima dello scalamento della catena; cambio settimana dai bordi 1400 ms e mai prima della settimana corrente
- ScheduleService.isFrozen (confermata o passata): non trascinabile, non scalabile, non sovrascrivibile; si libera solo cancellandola dal direttore
- Export Excel PS: fill dei sottomoduli schiariti (pastello, ~82% bianco), testo nero, leggibili in stampa B/N; template rigenerato con tools/rederive_ps_blank.py

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/assets/templates/ps_weekly_blank.xlsx
+++ b/assets/templates/ps_weekly_blank.xlsx
@@ -3494,121 +3494,121 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF6366F1"/>
+        <fgColor rgb="FFE3E3FC"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF3B82F6"/>
+        <fgColor rgb="FFDCE8FD"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF06B6D4"/>
+        <fgColor rgb="FFD2F2F7"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF14B8A6"/>
+        <fgColor rgb="FFD5F2EF"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF22C55E"/>
+        <fgColor rgb="FFD7F5E2"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF84CC16"/>
+        <fgColor rgb="FFE9F6D5"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFF59E0B"/>
+        <fgColor rgb="FFFDEED3"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFF97316"/>
+        <fgColor rgb="FFFEE6D5"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFEF4444"/>
+        <fgColor rgb="FFFCDDDD"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFEC4899"/>
+        <fgColor rgb="FFFCDEED"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFA855F7"/>
+        <fgColor rgb="FFEFE0FE"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF8B5CF6"/>
+        <fgColor rgb="FFEAE2FD"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF0EA5E9"/>
+        <fgColor rgb="FFD4EFFB"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF10B981"/>
+        <fgColor rgb="FFD4F2E8"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFD97706"/>
+        <fgColor rgb="FFF8E7D2"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF64748B"/>
+        <fgColor rgb="FFE3E6EA"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF78716C"/>
+        <fgColor rgb="FFE7E5E5"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF854D0E"/>
+        <fgColor rgb="FFE9DFD4"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF166534"/>
+        <fgColor rgb="FFD5E3DA"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF6B7280"/>
+        <fgColor rgb="FFE4E6E8"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>

</xml_diff>

<commit_message>
feat(corsi): planner recuperi visibili, svalida lezioni, OJT con deroga, bordi Excel PS
- Planner: icona nota su cella vuota più grande; menu "Impostazioni" solo icona,
  invio notifiche come pulsante separato nell'header.
- Svalida di una singola lezione e di un'intera giornata (direttore); gli appelli
  restano registrati.
- Recuperi: scelta teoria/pratica quando servono entrambe, riga "Rec." nel planner
  (anche per quelli già registrati, più persone e più moduli nello stesso periodo),
  validazione e svalidazione; i recuperi non validati non contano nelle statistiche.
- OJT: l'istruttore in OJT è GO anche per le 35 h entro 2 anni da ojtAt e per le 6 h
  entro 1 anno; scaduto il termine senza ore diventa NO GO (GradeService.ojtGraceFor,
  test/ojt_grace_test.dart).
- Excel PS: bordo destro esplicito (colonna O) su tutte le righe della tabella
  studenti; template rigenerato.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/assets/templates/ps_weekly_blank.xlsx
+++ b/assets/templates/ps_weekly_blank.xlsx
@@ -13892,7 +13892,7 @@
       <c r="L49" s="1220"/>
       <c r="M49" s="1220"/>
       <c r="N49" s="1220"/>
-      <c r="O49" s="1220"/>
+      <c r="O49" s="1221"/>
       <c r="P49" s="488"/>
     </row>
     <row r="50" spans="2:16" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -13909,7 +13909,7 @@
       <c r="L50" s="1224"/>
       <c r="M50" s="1224"/>
       <c r="N50" s="1224"/>
-      <c r="O50" s="1224"/>
+      <c r="O50" s="1256"/>
       <c r="P50" s="488"/>
     </row>
     <row r="51" spans="2:16" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -13942,7 +13942,7 @@
       <c r="L52" s="1216"/>
       <c r="M52" s="1216"/>
       <c r="N52" s="1216"/>
-      <c r="O52" s="1216"/>
+      <c r="O52" s="1217"/>
       <c r="P52" s="488"/>
     </row>
     <row r="53" spans="2:16" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -13975,7 +13975,7 @@
       <c r="L54" s="1216"/>
       <c r="M54" s="1216"/>
       <c r="N54" s="1216"/>
-      <c r="O54" s="1216"/>
+      <c r="O54" s="1217"/>
       <c r="P54" s="488"/>
     </row>
     <row r="55" spans="2:16" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -13991,7 +13991,7 @@
       <c r="L55" s="1216"/>
       <c r="M55" s="1216"/>
       <c r="N55" s="1216"/>
-      <c r="O55" s="1216"/>
+      <c r="O55" s="1217"/>
       <c r="P55" s="488"/>
     </row>
     <row r="56" spans="2:16" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -14008,7 +14008,7 @@
       <c r="L56" s="1216"/>
       <c r="M56" s="1216"/>
       <c r="N56" s="1216"/>
-      <c r="O56" s="1216"/>
+      <c r="O56" s="1217"/>
       <c r="P56" s="488"/>
     </row>
     <row r="57" spans="2:16" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
@@ -14025,7 +14025,7 @@
       <c r="L57" s="1216"/>
       <c r="M57" s="1216"/>
       <c r="N57" s="1216"/>
-      <c r="O57" s="1216"/>
+      <c r="O57" s="1217"/>
       <c r="P57" s="488"/>
     </row>
     <row r="58" spans="2:16" ht="14.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
feat(corsi): azioni giornata affiancate, deroga OJT anche per OJT chiusi, Excel PS lista unica
- Planner: le tre azioni dell'header di giornata (Assenti, Valida N, Svalida N) sono
  affiancate; se i testi non entrano restano solo le icone (con tooltip).
- OJT: la deroga (GO sulle 6 h per 1 anno e sulle 35 h per 2 anni) vale anche per gli
  OJT già chiusi. Per i dati legacy senza ojt_at l'ancora è la data dell'ultimo update
  'ojt' (GradeService.ojtGraceFor con lastOjt). "Modifica OJT" disponibile anche per
  chi ha solo l'update storico.
- Excel PS: nessuna distinzione Esercito/Carabinieri. Un'unica lista frequentatori
  ordinata per cognome (9 righe a sinistra, poi 9 a destra, numerazione continua,
  max 18), senza grado. Intestazioni del template neutre "NOME e COGNOME", modello
  generale per tutti i corsi (tools/rederive_ps_blank.py aggiornato, template
  rigenerato).

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/assets/templates/ps_weekly_blank.xlsx
+++ b/assets/templates/ps_weekly_blank.xlsx
@@ -2243,10 +2243,10 @@
     <t>C.le Magg. FERDINANDO AVELLO</t>
   </si>
   <si>
-    <t>GRADO, NOME e COGNOME (ESERCITO)</t>
-  </si>
-  <si>
-    <t>GRADO, NOME e COGNOME (CARABINIERI)</t>
+    <t>NOME e COGNOME</t>
+  </si>
+  <si>
+    <t>NOME e COGNOME</t>
   </si>
   <si>
     <t>C.le Magg. OSKAR FONTANA</t>

</xml_diff>

<commit_message>
fix(excel PS): bordi pausa pranzo uniformi lun-gio
Riga 39 (giovedì) senza bordo sopra, C23 senza top, C31/N31 senza lato:
rederive_ps_blank.py rimappa gli stili 66_PS delle righe pranzo agli xf
equivalenti con griglia sottile completa (LUNCH_FULL_BORDER). Test: righe
23/31/39 con gli stessi bordi della 15.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/assets/templates/ps_weekly_blank.xlsx
+++ b/assets/templates/ps_weekly_blank.xlsx
@@ -13186,7 +13186,7 @@
     </row>
     <row r="23" spans="2:33" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B23" s="614"/>
-      <c r="C23" s="550" t="s">
+      <c r="C23" s="540" t="s">
         <v>671</v>
       </c>
       <c r="D23" s="653"/>
@@ -13381,7 +13381,7 @@
     </row>
     <row r="31" spans="2:33" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B31" s="614"/>
-      <c r="C31" s="583" t="s">
+      <c r="C31" s="540" t="s">
         <v>671</v>
       </c>
       <c r="D31" s="653"/>
@@ -13394,7 +13394,7 @@
       <c r="K31" s="576"/>
       <c r="L31" s="576"/>
       <c r="M31" s="576"/>
-      <c r="N31" s="1249"/>
+      <c r="N31" s="1230"/>
       <c r="O31" s="1231"/>
       <c r="Q31" s="531"/>
       <c r="S31" s="531"/>
@@ -13595,19 +13595,19 @@
     </row>
     <row r="39" spans="1:29" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B39" s="614"/>
-      <c r="C39" s="550" t="s">
+      <c r="C39" s="540" t="s">
         <v>671</v>
       </c>
-      <c r="D39" s="1236"/>
-      <c r="E39" s="1237"/>
-      <c r="F39" s="1238"/>
-      <c r="G39" s="566"/>
-      <c r="H39" s="551"/>
-      <c r="I39" s="1254"/>
-      <c r="J39" s="1254"/>
-      <c r="K39" s="578"/>
-      <c r="L39" s="566"/>
-      <c r="M39" s="566"/>
+      <c r="D39" s="653"/>
+      <c r="E39" s="653"/>
+      <c r="F39" s="653"/>
+      <c r="G39" s="567"/>
+      <c r="H39" s="568"/>
+      <c r="I39" s="654"/>
+      <c r="J39" s="654"/>
+      <c r="K39" s="567"/>
+      <c r="L39" s="567"/>
+      <c r="M39" s="567"/>
       <c r="N39" s="1230"/>
       <c r="O39" s="1231"/>
       <c r="AB39" s="531"/>

</xml_diff>